<commit_message>
fix 4 issues stated and cleaned repo
</commit_message>
<xml_diff>
--- a/data/data/ICICI Prudential Mutual Fund/BHARAT 22 ETF.xlsx
+++ b/data/data/ICICI Prudential Mutual Fund/BHARAT 22 ETF.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="95">
   <si>
     <t>ICICI Prudential Mutual Fund</t>
   </si>
@@ -22,7 +22,7 @@
     <t>BHARAT 22 ETF</t>
   </si>
   <si>
-    <t>Portfolio as on Jan 31,2025</t>
+    <t>Portfolio as on May 31,2025</t>
   </si>
   <si>
     <t>Company/Issuer/Instrument Name</t>
@@ -61,6 +61,15 @@
     <t>Listed / Awaiting Listing On Stock Exchanges</t>
   </si>
   <si>
+    <t>Larsen &amp; Toubro Ltd.</t>
+  </si>
+  <si>
+    <t>INE018A01030</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
     <t>ITC Ltd.</t>
   </si>
   <si>
@@ -70,15 +79,6 @@
     <t>Diversified Fmcg</t>
   </si>
   <si>
-    <t>Larsen &amp; Toubro Ltd.</t>
-  </si>
-  <si>
-    <t>INE018A01030</t>
-  </si>
-  <si>
-    <t>Construction</t>
-  </si>
-  <si>
     <t>NTPC Ltd.</t>
   </si>
   <si>
@@ -88,25 +88,52 @@
     <t>Power</t>
   </si>
   <si>
+    <t>Axis Bank Ltd.</t>
+  </si>
+  <si>
+    <t>INE238A01034</t>
+  </si>
+  <si>
+    <t>Banks</t>
+  </si>
+  <si>
+    <t>State Bank Of India</t>
+  </si>
+  <si>
+    <t>INE062A01020</t>
+  </si>
+  <si>
     <t>Power Grid Corporation Of India Ltd.</t>
   </si>
   <si>
     <t>INE752E01010</t>
   </si>
   <si>
-    <t>State Bank Of India</t>
-  </si>
-  <si>
-    <t>INE062A01020</t>
-  </si>
-  <si>
-    <t>Banks</t>
-  </si>
-  <si>
-    <t>Axis Bank Ltd.</t>
-  </si>
-  <si>
-    <t>INE238A01034</t>
+    <t>Bharat Electronics Ltd.</t>
+  </si>
+  <si>
+    <t>INE263A01024</t>
+  </si>
+  <si>
+    <t>Aerospace &amp; Defense</t>
+  </si>
+  <si>
+    <t>Oil &amp; Natural Gas Corporation Ltd.</t>
+  </si>
+  <si>
+    <t>INE213A01029</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>Coal India Ltd.</t>
+  </si>
+  <si>
+    <t>INE522F01014</t>
+  </si>
+  <si>
+    <t>Consumable Fuels</t>
   </si>
   <si>
     <t>National Aluminium Company Ltd.</t>
@@ -118,33 +145,6 @@
     <t>Non - Ferrous Metals</t>
   </si>
   <si>
-    <t>Bharat Electronics Ltd.</t>
-  </si>
-  <si>
-    <t>INE263A01024</t>
-  </si>
-  <si>
-    <t>Aerospace &amp; Defense</t>
-  </si>
-  <si>
-    <t>Oil &amp; Natural Gas Corporation Ltd.</t>
-  </si>
-  <si>
-    <t>INE213A01029</t>
-  </si>
-  <si>
-    <t>Oil</t>
-  </si>
-  <si>
-    <t>Coal India Ltd.</t>
-  </si>
-  <si>
-    <t>INE522F01014</t>
-  </si>
-  <si>
-    <t>Consumable Fuels</t>
-  </si>
-  <si>
     <t>Bharat Petroleum Corporation Ltd.</t>
   </si>
   <si>
@@ -169,6 +169,12 @@
     <t>Gas</t>
   </si>
   <si>
+    <t>NHPC Ltd.</t>
+  </si>
+  <si>
+    <t>INE848E01016</t>
+  </si>
+  <si>
     <t>Power Finance Corporation Ltd.</t>
   </si>
   <si>
@@ -184,25 +190,16 @@
     <t>INE020B01018</t>
   </si>
   <si>
-    <t>NHPC Ltd.</t>
-  </si>
-  <si>
-    <t>INE848E01016</t>
-  </si>
-  <si>
     <t>Bank Of Baroda</t>
   </si>
   <si>
     <t>INE028A01039</t>
   </si>
   <si>
-    <t>ITC Hotels Ltd</t>
-  </si>
-  <si>
-    <t>INE379A01028</t>
-  </si>
-  <si>
-    <t>Leisure Services</t>
+    <t>Indian Bank</t>
+  </si>
+  <si>
+    <t>INE562A01011</t>
   </si>
   <si>
     <t>NBCC (India) Ltd.</t>
@@ -211,10 +208,10 @@
     <t>INE095N01031</t>
   </si>
   <si>
-    <t>Indian Bank</t>
-  </si>
-  <si>
-    <t>INE562A01011</t>
+    <t>NLC India Ltd.</t>
+  </si>
+  <si>
+    <t>INE589A01014</t>
   </si>
   <si>
     <t>SJVN Ltd.</t>
@@ -223,12 +220,6 @@
     <t>INE002L01015</t>
   </si>
   <si>
-    <t>NLC India Ltd.</t>
-  </si>
-  <si>
-    <t>INE589A01014</t>
-  </si>
-  <si>
     <t>Engineers India Ltd.</t>
   </si>
   <si>
@@ -298,7 +289,7 @@
     <t>@ As per AMFI Best Practices Guidelines Circular No. 91/ 2020 - 21 dated March 24, 2021 on Valuation of AT-1 Bonds and Tier 2 Bonds, Yield to call is disclosed for AT-1 Bonds and Tier 2 Bonds issued by Banks as provided by Valuation agencies.</t>
   </si>
   <si>
-    <t>For Instances of Deviation In valuation Of Securities as per SEBI master circular ref no SEBI/HO/IMD/IMD-PoD-1/P/CIR/2023/74 dated May 19, 2023.Refer link: https://www.icicipruamc.com/statutory-disclosures/deviation-in-valuation-of-securities</t>
+    <t>For Instances of Deviation In valuation Of Securities as per SEBI master circular ref no SEBI/HO/IMD/IMD-PoD-1/P/CIR/2024/90 dated June 27, 2024. Refer link: https://www.icicipruamc.com/about-us/statutory-disclosures?currentTabFilter=OtherDisclosures&amp;&amp;subCatTabFilter=deviationinvaluationofsecurities</t>
   </si>
   <si>
     <t>As per AMFI Best Practices Guidelines Circular No. AMFI/ 35P/ MEM-COR/ 72 / 2022-23 dated December 31, 2022 on Standard format for disclosure Portfolio YTM for Debt Schemes, Yield of the instrument is disclosed on annualized basis as provided by Valuation agencies.</t>
@@ -308,9 +299,6 @@
   </si>
   <si>
     <t>Benchmark Riskometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark name - BSE Bharat 22 TRI </t>
   </si>
 </sst>
 </file>
@@ -536,7 +524,7 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -629,9 +617,6 @@
       <protection/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyBorder="1" applyProtection="1">
-      <protection/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
       <protection/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1125,19 +1110,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="B1:J90"/>
+  <dimension ref="B1:J89"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="27" width="10.0" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="27" width="53.57142857142857" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="27" width="16.285714285714285" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="27" width="9.714285714285714" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="27" width="22.571428571428573" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="27" width="11.142857142857142" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="27" width="38.714285714285715" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="27" width="11.714285714285714" collapsed="true"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="27" width="29.714285714285715" collapsed="true"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="27" width="26.714285714285715" collapsed="true"/>
+    <col min="1" max="1" customWidth="true" style="26" width="10.0" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="26" width="53.57142857142857" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="26" width="16.285714285714285" collapsed="true"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="26" width="9.714285714285714" collapsed="true"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="26" width="22.571428571428573" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="26" width="11.142857142857142" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="26" width="38.714285714285715" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="26" width="11.714285714285714" collapsed="true"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="26" width="29.714285714285715" collapsed="true"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="26" width="26.714285714285715" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="15" customHeight="1">
@@ -1225,10 +1210,10 @@
         <v>13</v>
       </c>
       <c r="G5" s="9">
-        <v>1790573.3699999996</v>
+        <v>1743152.05</v>
       </c>
       <c r="H5" s="10">
-        <v>0.9982112588882999</v>
+        <v>0.9975267616535999</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>13</v>
@@ -1262,10 +1247,10 @@
         <v>13</v>
       </c>
       <c r="G7" s="9">
-        <v>1790573.3699999996</v>
+        <v>1743152.05</v>
       </c>
       <c r="H7" s="10">
-        <v>0.9982112588882999</v>
+        <v>0.9975267616535999</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>13</v>
@@ -1288,13 +1273,13 @@
         <v>17</v>
       </c>
       <c r="F8" s="14">
-        <v>66182477</v>
+        <v>7430927</v>
       </c>
       <c r="G8" s="15">
-        <v>296199.68</v>
+        <v>273142.30</v>
       </c>
       <c r="H8" s="16">
-        <v>0.1651257973614</v>
+        <v>0.1563069348941</v>
       </c>
       <c r="I8" s="15" t="s">
         <v>13</v>
@@ -1317,13 +1302,13 @@
         <v>20</v>
       </c>
       <c r="F9" s="14">
-        <v>7405377</v>
+        <v>57591940</v>
       </c>
       <c r="G9" s="15">
-        <v>264164.61</v>
+        <v>240676.72</v>
       </c>
       <c r="H9" s="16">
-        <v>0.1472668433028</v>
+        <v>0.1377283577226</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>13</v>
@@ -1346,13 +1331,13 @@
         <v>23</v>
       </c>
       <c r="F10" s="14">
-        <v>50703784</v>
+        <v>47524752</v>
       </c>
       <c r="G10" s="15">
-        <v>164407.02</v>
+        <v>158851.48</v>
       </c>
       <c r="H10" s="16">
-        <v>0.0916538473955</v>
+        <v>0.0909034885559</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>13</v>
@@ -1372,16 +1357,16 @@
         <v>13</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F11" s="14">
-        <v>48632808</v>
+        <v>12388948</v>
       </c>
       <c r="G11" s="15">
-        <v>146798.13</v>
+        <v>147682.45</v>
       </c>
       <c r="H11" s="16">
-        <v>0.0818372196331</v>
+        <v>0.0845119598727</v>
       </c>
       <c r="I11" s="15" t="s">
         <v>13</v>
@@ -1392,25 +1377,25 @@
     </row>
     <row r="12" spans="2:10" ht="15" customHeight="1">
       <c r="B12" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>28</v>
-      </c>
       <c r="F12" s="14">
-        <v>17018202</v>
+        <v>16690214</v>
       </c>
       <c r="G12" s="15">
-        <v>131567.72</v>
+        <v>135591.3</v>
       </c>
       <c r="H12" s="16">
-        <v>0.0733465501111</v>
+        <v>0.077592743787</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>13</v>
@@ -1430,16 +1415,16 @@
         <v>13</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F13" s="14">
-        <v>12575417</v>
+        <v>45583595</v>
       </c>
       <c r="G13" s="15">
-        <v>124043.91</v>
+        <v>132146.84</v>
       </c>
       <c r="H13" s="16">
-        <v>0.0691521663581</v>
+        <v>0.075621635742</v>
       </c>
       <c r="I13" s="15" t="s">
         <v>13</v>
@@ -1462,13 +1447,13 @@
         <v>33</v>
       </c>
       <c r="F14" s="14">
-        <v>55213006</v>
+        <v>25402810</v>
       </c>
       <c r="G14" s="15">
-        <v>111640.70</v>
+        <v>97699.21</v>
       </c>
       <c r="H14" s="16">
-        <v>0.0622376081077</v>
+        <v>0.0559088213604</v>
       </c>
       <c r="I14" s="15" t="s">
         <v>13</v>
@@ -1491,13 +1476,13 @@
         <v>36</v>
       </c>
       <c r="F15" s="14">
-        <v>35680324</v>
+        <v>39150628</v>
       </c>
       <c r="G15" s="15">
-        <v>104471.99</v>
+        <v>93746.18</v>
       </c>
       <c r="H15" s="16">
-        <v>0.0582411859819</v>
+        <v>0.0536466817985</v>
       </c>
       <c r="I15" s="15" t="s">
         <v>13</v>
@@ -1520,13 +1505,13 @@
         <v>39</v>
       </c>
       <c r="F16" s="14">
-        <v>35574859</v>
+        <v>22890827</v>
       </c>
       <c r="G16" s="15">
-        <v>93384</v>
+        <v>90933.81</v>
       </c>
       <c r="H16" s="16">
-        <v>0.0520598383522</v>
+        <v>0.0520372901573</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>13</v>
@@ -1549,13 +1534,13 @@
         <v>42</v>
       </c>
       <c r="F17" s="14">
-        <v>20800133</v>
+        <v>41301033</v>
       </c>
       <c r="G17" s="15">
-        <v>82326.93</v>
+        <v>74507.06</v>
       </c>
       <c r="H17" s="16">
-        <v>0.0458957280459</v>
+        <v>0.0426370070713</v>
       </c>
       <c r="I17" s="15" t="s">
         <v>13</v>
@@ -1578,13 +1563,13 @@
         <v>45</v>
       </c>
       <c r="F18" s="14">
-        <v>17413422</v>
+        <v>19599084</v>
       </c>
       <c r="G18" s="15">
-        <v>45483.86</v>
+        <v>62354.49</v>
       </c>
       <c r="H18" s="16">
-        <v>0.0253564036584</v>
+        <v>0.0356826431086</v>
       </c>
       <c r="I18" s="15" t="s">
         <v>13</v>
@@ -1607,13 +1592,13 @@
         <v>45</v>
       </c>
       <c r="F19" s="14">
-        <v>34779881</v>
+        <v>36858095</v>
       </c>
       <c r="G19" s="15">
-        <v>44709.54</v>
+        <v>52320.07</v>
       </c>
       <c r="H19" s="16">
-        <v>0.0249247346997</v>
+        <v>0.0299404002058</v>
       </c>
       <c r="I19" s="15" t="s">
         <v>13</v>
@@ -1636,13 +1621,13 @@
         <v>50</v>
       </c>
       <c r="F20" s="14">
-        <v>24591081</v>
+        <v>27062816</v>
       </c>
       <c r="G20" s="15">
-        <v>43575.40</v>
+        <v>51365.22</v>
       </c>
       <c r="H20" s="16">
-        <v>0.0242924728019</v>
+        <v>0.0293939829106</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>13</v>
@@ -1662,16 +1647,16 @@
         <v>13</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="F21" s="14">
-        <v>6439256</v>
+        <v>31146875</v>
       </c>
       <c r="G21" s="15">
-        <v>27209.08</v>
+        <v>27213.02</v>
       </c>
       <c r="H21" s="16">
-        <v>0.0151685546401</v>
+        <v>0.0155727756023</v>
       </c>
       <c r="I21" s="15" t="s">
         <v>13</v>
@@ -1682,25 +1667,25 @@
     </row>
     <row r="22" spans="2:10" ht="15" customHeight="1">
       <c r="B22" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="D22" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>53</v>
-      </c>
       <c r="F22" s="14">
-        <v>5488336</v>
+        <v>6315151</v>
       </c>
       <c r="G22" s="15">
-        <v>24689.28</v>
+        <v>25626.88</v>
       </c>
       <c r="H22" s="16">
-        <v>0.0137638131353</v>
+        <v>0.014665099707</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>13</v>
@@ -1720,16 +1705,16 @@
         <v>13</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="F23" s="14">
-        <v>28942597</v>
+        <v>5382566</v>
       </c>
       <c r="G23" s="15">
-        <v>23287.21</v>
+        <v>21691.74</v>
       </c>
       <c r="H23" s="16">
-        <v>0.0129821852595</v>
+        <v>0.0124131977797</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>13</v>
@@ -1749,16 +1734,16 @@
         <v>13</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F24" s="14">
-        <v>8255887</v>
+        <v>8096758</v>
       </c>
       <c r="G24" s="15">
-        <v>17618.06</v>
+        <v>20217.60</v>
       </c>
       <c r="H24" s="16">
-        <v>0.0098217398663</v>
+        <v>0.0115696143984</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>13</v>
@@ -1778,16 +1763,16 @@
         <v>13</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F25" s="14">
-        <v>6618246</v>
+        <v>1523116</v>
       </c>
       <c r="G25" s="15">
-        <v>10896.94</v>
+        <v>9407.53</v>
       </c>
       <c r="H25" s="16">
-        <v>0.0060748408178</v>
+        <v>0.0053835022229</v>
       </c>
       <c r="I25" s="15" t="s">
         <v>13</v>
@@ -1798,25 +1783,25 @@
     </row>
     <row r="26" spans="2:10" ht="15" customHeight="1">
       <c r="B26" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>64</v>
-      </c>
       <c r="D26" s="13" t="s">
         <v>13</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F26" s="14">
-        <v>10220579</v>
+        <v>7276605</v>
       </c>
       <c r="G26" s="15">
-        <v>10201.16</v>
+        <v>8977.15</v>
       </c>
       <c r="H26" s="16">
-        <v>0.0056869564444</v>
+        <v>0.0051372152924</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>13</v>
@@ -1827,25 +1812,25 @@
     </row>
     <row r="27" spans="2:10" ht="15" customHeight="1">
       <c r="B27" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>66</v>
-      </c>
       <c r="D27" s="13" t="s">
         <v>13</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F27" s="14">
-        <v>1553050</v>
+        <v>3190009</v>
       </c>
       <c r="G27" s="15">
-        <v>8632.63</v>
+        <v>7711.85</v>
       </c>
       <c r="H27" s="16">
-        <v>0.0048125302231</v>
+        <v>0.0044131415597</v>
       </c>
       <c r="I27" s="15" t="s">
         <v>13</v>
@@ -1856,10 +1841,10 @@
     </row>
     <row r="28" spans="2:10" ht="15" customHeight="1">
       <c r="B28" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>67</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>68</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>13</v>
@@ -1868,13 +1853,13 @@
         <v>23</v>
       </c>
       <c r="F28" s="14">
-        <v>5451740</v>
+        <v>7075281</v>
       </c>
       <c r="G28" s="15">
-        <v>5309.99</v>
+        <v>6816.33</v>
       </c>
       <c r="H28" s="16">
-        <v>0.0029602203916</v>
+        <v>0.0039006761293</v>
       </c>
       <c r="I28" s="15" t="s">
         <v>13</v>
@@ -1885,25 +1870,25 @@
     </row>
     <row r="29" spans="2:10" ht="15" customHeight="1">
       <c r="B29" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="13" t="s">
-        <v>70</v>
-      </c>
       <c r="D29" s="13" t="s">
         <v>13</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F29" s="14">
-        <v>2367583</v>
+        <v>1953198</v>
       </c>
       <c r="G29" s="15">
-        <v>5256.03</v>
+        <v>4472.82</v>
       </c>
       <c r="H29" s="16">
-        <v>0.002930138698</v>
+        <v>0.0025595917751</v>
       </c>
       <c r="I29" s="15" t="s">
         <v>13</v>
@@ -1914,708 +1899,682 @@
     </row>
     <row r="30" spans="2:10" ht="15" customHeight="1">
       <c r="B30" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" ht="15" customHeight="1">
+      <c r="B31" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="H31" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" ht="15" customHeight="1">
+      <c r="B32" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" ht="15" customHeight="1">
+      <c r="B33" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="14">
-        <v>2743430</v>
-      </c>
-      <c r="G30" s="15">
-        <v>4699.50</v>
-      </c>
-      <c r="H30" s="16">
-        <v>0.0026198836025</v>
-      </c>
-      <c r="I30" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="J30" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="2:10" ht="15" customHeight="1">
-      <c r="B31" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J31" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="2:10" ht="15" customHeight="1">
-      <c r="B32" s="7" t="s">
+      <c r="C33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I33" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" ht="15" customHeight="1">
+      <c r="B34" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J34" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" ht="15" customHeight="1">
+      <c r="B35" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I35" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J35" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" ht="15" customHeight="1">
+      <c r="B36" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J36" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" ht="15" customHeight="1">
+      <c r="B37" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="9" t="s">
+      <c r="C37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J37" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" ht="15" customHeight="1">
+      <c r="B38" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J38" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" ht="15" customHeight="1">
+      <c r="B39" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="H32" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J32" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="2:10" ht="15" customHeight="1">
-      <c r="B33" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J33" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="2:10" ht="15" customHeight="1">
-      <c r="B34" s="7" t="s">
+      <c r="C39" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I39" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J39" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" ht="15" customHeight="1">
+      <c r="B40" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J40" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" ht="15" customHeight="1">
+      <c r="B41" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J34" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="2:10" ht="15" customHeight="1">
-      <c r="B35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J35" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="2:10" ht="15" customHeight="1">
-      <c r="B36" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J36" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" ht="15" customHeight="1">
-      <c r="B37" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J37" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" ht="15" customHeight="1">
-      <c r="B38" s="7" t="s">
+      <c r="C41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I41" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J41" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" ht="15" customHeight="1">
+      <c r="B42" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J42" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" ht="15" customHeight="1">
+      <c r="B43" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H38" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I38" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J38" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="2:10" ht="15" customHeight="1">
-      <c r="B39" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J39" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" ht="15" customHeight="1">
-      <c r="B40" s="7" t="s">
+      <c r="C43" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I43" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J43" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" ht="15" customHeight="1">
+      <c r="B44" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J44" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" ht="15" customHeight="1">
+      <c r="B45" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C40" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G40" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H40" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I40" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J40" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" ht="15" customHeight="1">
-      <c r="B41" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J41" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="2:10" ht="15" customHeight="1">
-      <c r="B42" s="7" t="s">
+      <c r="C45" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I45" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J45" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" ht="15" customHeight="1">
+      <c r="B46" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J46" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" ht="15" customHeight="1">
+      <c r="B47" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H42" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I42" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J42" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="2:10" ht="15" customHeight="1">
-      <c r="B43" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J43" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="2:10" ht="15" customHeight="1">
-      <c r="B44" s="7" t="s">
+      <c r="C47" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I47" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J47" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" ht="15" customHeight="1">
+      <c r="B48" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J48" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" ht="15" customHeight="1">
+      <c r="B49" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C44" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I44" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J44" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="2:10" ht="15" customHeight="1">
-      <c r="B45" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J45" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" ht="15" customHeight="1">
-      <c r="B46" s="7" t="s">
+      <c r="C49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I49" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J49" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" ht="15" customHeight="1">
+      <c r="B50" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" ht="15" customHeight="1">
+      <c r="B51" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C46" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H46" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I46" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J46" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" ht="15" customHeight="1">
-      <c r="B47" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J47" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="2:10" ht="15" customHeight="1">
-      <c r="B48" s="7" t="s">
+      <c r="C51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I51" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" ht="15" customHeight="1">
+      <c r="B52" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" ht="15" customHeight="1">
+      <c r="B53" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C48" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H48" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I48" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J48" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="2:10" ht="15" customHeight="1">
-      <c r="B49" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J49" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="50" spans="2:10" ht="15" customHeight="1">
-      <c r="B50" s="7" t="s">
+      <c r="C53" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I53" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" ht="15" customHeight="1">
+      <c r="B54" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J54" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10" ht="15" customHeight="1">
+      <c r="B55" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C50" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H50" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I50" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J50" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" spans="2:10" ht="15" customHeight="1">
-      <c r="B51" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J51" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="52" spans="2:10" ht="15" customHeight="1">
-      <c r="B52" s="7" t="s">
+      <c r="C55" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H55" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I55" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J55" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="2:10" ht="15" customHeight="1">
+      <c r="B56" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J56" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" ht="15" customHeight="1">
+      <c r="B57" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C52" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H52" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I52" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J52" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="2:10" ht="15" customHeight="1">
-      <c r="B53" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J53" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="2:10" ht="15" customHeight="1">
-      <c r="B54" s="7" t="s">
+      <c r="C57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" s="9">
+        <v>2704.83</v>
+      </c>
+      <c r="H57" s="10">
+        <v>0.0015478513826</v>
+      </c>
+      <c r="I57" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J57" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="2:10" ht="15" customHeight="1">
+      <c r="B58" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J58" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="2:10" ht="15" customHeight="1">
+      <c r="B59" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C54" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D54" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H54" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I54" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J54" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="2:10" ht="15" customHeight="1">
-      <c r="B55" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J55" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="2:10" ht="15" customHeight="1">
-      <c r="B56" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="C56" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H56" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I56" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J56" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="2:10" ht="15" customHeight="1">
-      <c r="B57" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J57" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="58" spans="2:10" ht="15" customHeight="1">
-      <c r="B58" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C58" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" s="9">
-        <v>137.97</v>
-      </c>
-      <c r="H58" s="10">
-        <v>0.0000769157018</v>
-      </c>
-      <c r="I58" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J58" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="59" spans="2:10" ht="15" customHeight="1">
-      <c r="B59" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J59" s="11" t="s">
+      <c r="C59" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="18">
+        <v>1617.0896286997013</v>
+      </c>
+      <c r="H59" s="19">
+        <v>0.0009253869624411615</v>
+      </c>
+      <c r="I59" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="J59" s="20" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="60" spans="2:10" ht="15" customHeight="1">
       <c r="B60" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C60" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" s="18">
+        <v>1747473.9696287</v>
+      </c>
+      <c r="H60" s="19">
+        <v>0.9999999999986411</v>
+      </c>
+      <c r="I60" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="J60" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="2:3" ht="15" customHeight="1">
+      <c r="B62" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C62" s="22"/>
+    </row>
+    <row r="63" spans="2:3" ht="15" customHeight="1">
+      <c r="B63" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G60" s="18">
-        <v>3070.6415740002412</v>
-      </c>
-      <c r="H60" s="19">
-        <v>0.001711825408852545</v>
-      </c>
-      <c r="I60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="J60" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="2:10" ht="15" customHeight="1">
-      <c r="B61" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C61" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D61" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E61" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F61" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G61" s="18">
-        <v>1793781.981574</v>
-      </c>
-      <c r="H61" s="19">
-        <v>0.9999999999989523</v>
-      </c>
-      <c r="I61" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="J61" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="2:3" ht="15" customHeight="1">
-      <c r="B63" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="C63" s="22"/>
+      <c r="C63" s="24" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="64" spans="2:3" ht="15" customHeight="1">
-      <c r="B64" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C64" s="24" t="s">
-        <v>7</v>
+      <c r="B64" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="C64" s="25">
+        <v>150000</v>
       </c>
     </row>
     <row r="65" spans="2:3" ht="15" customHeight="1">
       <c r="B65" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="C65" s="26">
-        <v>1080000</v>
+        <v>66</v>
+      </c>
+      <c r="C65" s="25">
+        <v>650000</v>
       </c>
     </row>
     <row r="67" spans="2:9" ht="15" customHeight="1">
       <c r="B67" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="27"/>
-      <c r="F67" s="27"/>
-      <c r="G67" s="27"/>
-      <c r="H67" s="27"/>
-      <c r="I67" s="27"/>
+        <v>88</v>
+      </c>
+      <c r="C67" s="26"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="26"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="26"/>
+      <c r="H67" s="26"/>
+      <c r="I67" s="26"/>
     </row>
     <row r="68" spans="2:8" ht="15" customHeight="1">
       <c r="B68" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C68" s="26"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="26"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="26"/>
+      <c r="H68" s="26"/>
+    </row>
+    <row r="69" spans="2:8" ht="27.6" customHeight="1">
+      <c r="B69" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C69" s="26"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
+      <c r="F69" s="26"/>
+      <c r="G69" s="26"/>
+      <c r="H69" s="26"/>
+    </row>
+    <row r="70" spans="2:8" ht="27.6" customHeight="1">
+      <c r="B70" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="C70" s="26"/>
+      <c r="D70" s="26"/>
+      <c r="E70" s="26"/>
+      <c r="F70" s="26"/>
+      <c r="G70" s="26"/>
+      <c r="H70" s="26"/>
+    </row>
+    <row r="71" spans="2:8" ht="27.6" customHeight="1">
+      <c r="B71" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="C68" s="27"/>
-      <c r="D68" s="27"/>
-      <c r="E68" s="27"/>
-      <c r="F68" s="27"/>
-      <c r="G68" s="27"/>
-      <c r="H68" s="27"/>
-    </row>
-    <row r="69" spans="2:8" ht="27.6" customHeight="1">
-      <c r="B69" s="28" t="s">
+      <c r="C71" s="26"/>
+      <c r="D71" s="26"/>
+      <c r="E71" s="26"/>
+      <c r="F71" s="26"/>
+      <c r="G71" s="26"/>
+      <c r="H71" s="26"/>
+    </row>
+    <row r="74" ht="15">
+      <c r="B74" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C69" s="27"/>
-      <c r="D69" s="27"/>
-      <c r="E69" s="27"/>
-      <c r="F69" s="27"/>
-      <c r="G69" s="27"/>
-      <c r="H69" s="27"/>
-    </row>
-    <row r="70" spans="2:8" ht="27.6" customHeight="1">
-      <c r="B70" s="28" t="s">
+    </row>
+    <row r="89" ht="15">
+      <c r="B89" s="26" t="s">
         <v>94</v>
-      </c>
-      <c r="C70" s="27"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="27"/>
-      <c r="F70" s="27"/>
-      <c r="G70" s="27"/>
-      <c r="H70" s="27"/>
-    </row>
-    <row r="71" spans="2:8" ht="27.6" customHeight="1">
-      <c r="B71" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="C71" s="27"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="27"/>
-      <c r="F71" s="27"/>
-      <c r="G71" s="27"/>
-      <c r="H71" s="27"/>
-    </row>
-    <row r="74" ht="15">
-      <c r="B74" s="27" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="89" ht="15">
-      <c r="B89" s="27" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="90" ht="15">
-      <c r="B90" s="27" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>